<commit_message>
Add Bloomberg update and portable export pipeline
</commit_message>
<xml_diff>
--- a/config/security_roots.xlsx
+++ b/config/security_roots.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Roots" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloomberg Update" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Security Roots'!$A$1:$L$7</definedName>
@@ -166,6 +167,18 @@
     <tableColumn id="10" name="aliases"/>
     <tableColumn id="11" name="product_group"/>
     <tableColumn id="12" name="sort_order"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BloombergUpdateSettings" displayName="BloombergUpdateSettings" ref="A1:C14" headerRowCount="1">
+  <autoFilter ref="A1:C14"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="setting"/>
+    <tableColumn id="2" name="value"/>
+    <tableColumn id="3" name="what it controls"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -460,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -518,48 +531,60 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Save the workbook, validate the Parquet, then rebuild the dashboard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Conversion checks</t>
+          <t>Review the Bloomberg Update sheet to control dates, fields, and connection settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Save the workbook, start the local dashboard, and press UPDATE DATA.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cpg → $/gal</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>divide by 100</t>
+          <t>Conversion checks</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>$/gal → $/bbl</t>
+          <t>cpg → $/gal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>multiply by gal_per_bbl</t>
+          <t>divide by 100</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>$/gal → $/bbl</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>multiply by gal_per_bbl</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>$/bbl → $/MT</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>multiply by bbl_per_mt</t>
         </is>
@@ -1000,4 +1025,246 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="82" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>what it controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>history_start</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2019-01-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Earliest observation date retained in the update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>contract_start_year</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>First delivery year included in the ticker universe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>contract_end_year</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2028</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Last delivery year included in the ticker universe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>contract_history_months</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>24</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Months of history requested before each delivery month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>reference_depth</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Maximum dated-contract reference retained, normally 1 or 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>overlap_days</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Days re-pulled for active contracts during an incremental update.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fields</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PX_LAST,PX_CLOSE,PX_SETTLE,PX_FAIR_1430</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bloomberg historical fields; PX_LAST is required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>localhost</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Bloomberg Desktop API host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>port</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8194</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bloomberg Desktop API port.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>//blp/refdata</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Bloomberg reference-data service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>batch_size</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>25</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Maximum securities sent in one Bloomberg request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>request_timeout_seconds</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>120</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Hard limit for each Bloomberg request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>standalone_max_mb</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>20</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Maximum portable HTML size before publication stops.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Make common names spreadsheet-authoritative
</commit_message>
<xml_diff>
--- a/config/security_roots.xlsx
+++ b/config/security_roots.xlsx
@@ -157,7 +157,7 @@
   <tableColumns count="12">
     <tableColumn id="1" name="enabled"/>
     <tableColumn id="2" name="root"/>
-    <tableColumn id="3" name="display_name"/>
+    <tableColumn id="3" name="common_name"/>
     <tableColumn id="4" name="yellow_key"/>
     <tableColumn id="5" name="native_unit"/>
     <tableColumn id="6" name="bbl_per_mt"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Add one row per Bloomberg root on the Security Roots sheet.</t>
+          <t>Add one row per Bloomberg root and set common_name to the label shown everywhere in the dashboard.</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>display_name</t>
+          <t>common_name</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Support adjustable Bloomberg ticker year formats
</commit_message>
<xml_diff>
--- a/config/security_roots.xlsx
+++ b/config/security_roots.xlsx
@@ -149,6 +149,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pricing Dashboard</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Examples: {root}{month_code}{y} {yellow_key} -&gt; HOG6 Comdty; use {yy} for HOG26 or {year} for HOG2026. Set yellow_key separately.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -473,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -547,44 +562,68 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ticker example</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HO + Feb (G) + {y} + Comdty produces HOG6 Comdty for 2026.</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Conversion checks</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>cpg → $/gal</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>divide by 100</t>
+          <t>Year placeholders</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Use {y} for 6, {yy} for 26, or {year} for 2026. yellow_key independently controls Comdty vs Index.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>$/gal → $/bbl</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>multiply by gal_per_bbl</t>
+          <t>Conversion checks</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>cpg → $/gal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>divide by 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>$/gal → $/bbl</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>multiply by gal_per_bbl</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>$/bbl → $/MT</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>multiply by bbl_per_mt</t>
         </is>
@@ -715,7 +754,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{root}{month_code}{yy} {yellow_key}</t>
+          <t>{root}{month_code}{y} {yellow_key}</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -769,7 +808,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>{root}{month_code}{yy} {yellow_key}</t>
+          <t>{root}{month_code}{y} {yellow_key}</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -823,7 +862,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>{root}{month_code}{yy} {yellow_key}</t>
+          <t>{root}{month_code}{y} {yellow_key}</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -877,7 +916,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>{root}{month_code}{yy} {yellow_key}</t>
+          <t>{root}{month_code}{y} {yellow_key}</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -931,7 +970,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>{root}{month_code}{yy} {yellow_key}</t>
+          <t>{root}{month_code}{y} {yellow_key}</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -985,7 +1024,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>{root}{month_code}{yy} {yellow_key}</t>
+          <t>{root}{month_code}{y} {yellow_key}</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1021,6 +1060,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Improve trade builder and add RVO flat curve
</commit_message>
<xml_diff>
--- a/config/security_roots.xlsx
+++ b/config/security_roots.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloomberg Update" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Security Roots'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Security Roots'!$A$1:$M$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -167,9 +167,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SecurityRoots" displayName="SecurityRoots" ref="A1:L7" headerRowCount="1">
-  <autoFilter ref="A1:L7"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SecurityRoots" displayName="SecurityRoots" ref="A1:M8" headerRowCount="1">
+  <autoFilter ref="A1:M8"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="enabled"/>
     <tableColumn id="2" name="root"/>
     <tableColumn id="3" name="common_name"/>
@@ -178,18 +178,19 @@
     <tableColumn id="6" name="bbl_per_mt"/>
     <tableColumn id="7" name="gal_per_bbl"/>
     <tableColumn id="8" name="ticker_template"/>
-    <tableColumn id="9" name="tradingview_symbol"/>
-    <tableColumn id="10" name="aliases"/>
-    <tableColumn id="11" name="product_group"/>
-    <tableColumn id="12" name="sort_order"/>
+    <tableColumn id="9" name="curve_mode"/>
+    <tableColumn id="10" name="tradingview_symbol"/>
+    <tableColumn id="11" name="aliases"/>
+    <tableColumn id="12" name="product_group"/>
+    <tableColumn id="13" name="sort_order"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BloombergUpdateSettings" displayName="BloombergUpdateSettings" ref="A1:C14" headerRowCount="1">
-  <autoFilter ref="A1:C14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BloombergUpdateSettings" displayName="BloombergUpdateSettings" ref="A1:C15" headerRowCount="1">
+  <autoFilter ref="A1:C15"/>
   <tableColumns count="3">
     <tableColumn id="1" name="setting"/>
     <tableColumn id="2" name="value"/>
@@ -488,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -522,7 +523,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Choose Comdty or Index and the native quote unit from the dropdowns.</t>
+          <t>Choose Comdty or Index, the native quote unit, and Monthly or Flat curve mode from the dropdowns.</t>
         </is>
       </c>
     </row>
@@ -546,7 +547,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Review the Bloomberg Update sheet to control dates, fields, and connection settings.</t>
+          <t>Review the Bloomberg Update sheet to control dates, full data fields, lightweight dashboard fields, and connection settings.</t>
         </is>
       </c>
     </row>
@@ -577,53 +578,65 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Flat example</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>RVO uses Flat with {root} {yellow_key}; Bloomberg pulls RVO Index once and the dashboard applies each daily value across the full curve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Year placeholders</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Use {y} for 6, {yy} for 26, or {year} for 2026. yellow_key independently controls Comdty vs Index.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Conversion checks</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cpg → $/gal</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>divide by 100</t>
+          <t>Conversion checks</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>$/gal → $/bbl</t>
+          <t>cpg → $/gal</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>multiply by gal_per_bbl</t>
+          <t>divide by 100</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>$/gal → $/bbl</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>multiply by gal_per_bbl</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>$/bbl → $/MT</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>multiply by bbl_per_mt</t>
         </is>
@@ -643,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -654,10 +667,11 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="43" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -703,20 +717,25 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
+          <t>curve_mode</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
           <t>tradingview_symbol</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>aliases</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>product_group</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
@@ -759,20 +778,25 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>NYMEX:WU</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>ME|GC JET</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Refined Products</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>10</v>
       </c>
     </row>
@@ -813,20 +837,25 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>NYMEX:HO</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>ULSD|HEATING OIL</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Refined Products</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -867,20 +896,25 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>NYMEX:RB</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>RBOB</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Refined Products</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>30</v>
       </c>
     </row>
@@ -890,22 +924,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>QS</t>
+          <t>RVO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ICE Low Sulphur Gasoil</t>
+          <t>RVO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Comdty</t>
+          <t>Index</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>$/MT</t>
+          <t>cpg</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -916,26 +950,27 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>{root}{month_code}{y} {yellow_key}</t>
+          <t>{root} {yellow_key}</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ICEEUR:QS1!</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>GASOIL|LSGO</t>
-        </is>
-      </c>
+          <t>Flat</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Refined Products</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>40</v>
+          <t>RENEWABLE VOLUME OBLIGATION</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Renewable Fuels</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -944,12 +979,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>QS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>WTI Crude Oil</t>
+          <t>ICE Low Sulphur Gasoil</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -959,11 +994,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$/bbl</t>
+          <t>$/MT</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.33</v>
+        <v>7.45</v>
       </c>
       <c r="G6" t="n">
         <v>42</v>
@@ -975,21 +1010,26 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NYMEX:CL</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>WTI</t>
+          <t>ICEEUR:QS1!</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Crude</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>50</v>
+          <t>GASOIL|LSGO</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Refined Products</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -998,12 +1038,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Brent Crude Oil</t>
+          <t>WTI Crude Oil</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1029,26 +1069,90 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>NYMEX:CL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>WTI</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Crude</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Brent Crude Oil</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Comdty</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>$/bbl</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="G8" t="n">
+        <v>42</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>{root}{month_code}{y} {yellow_key}</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>TVC:UKOIL</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>BRENT</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Crude</t>
         </is>
       </c>
-      <c r="L7" t="n">
+      <c r="M8" t="n">
         <v>60</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
-  <dataValidations count="3">
+  <autoFilter ref="A1:M8"/>
+  <dataValidations count="4">
     <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid value" error="Choose TRUE or FALSE" promptTitle="Pricing Dashboard" prompt="Choose TRUE or FALSE" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
@@ -1057,6 +1161,9 @@
     </dataValidation>
     <dataValidation sqref="E2:E501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid value" error="Choose the Bloomberg native quote unit" promptTitle="Pricing Dashboard" prompt="Choose the Bloomberg native quote unit" type="list">
       <formula1>"cpg,$/gal,$/bbl,$/MT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Invalid value" error="Monthly uses dated contracts; Flat uses one daily series with no month selector" promptTitle="Pricing Dashboard" prompt="Monthly uses dated contracts; Flat uses one daily series with no month selector" type="list">
+      <formula1>"Monthly,Flat"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1073,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1203,99 +1310,116 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bloomberg historical fields; PX_LAST is required.</t>
+          <t>Bloomberg fields retained in the full CSV and Parquet; PX_LAST is required.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>host</t>
+          <t>dashboard_fields</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>localhost</t>
+          <t>PX_LAST</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bloomberg Desktop API host.</t>
+          <t>Subset embedded in the portable dashboard; every value must also appear in fields.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>port</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>8194</v>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>localhost</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bloomberg Desktop API port.</t>
+          <t>Bloomberg Desktop API host.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>service</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>//blp/refdata</t>
-        </is>
+          <t>port</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8194</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bloomberg reference-data service.</t>
+          <t>Bloomberg Desktop API port.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>batch_size</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>25</v>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>//blp/refdata</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Maximum securities sent in one Bloomberg request.</t>
+          <t>Bloomberg reference-data service.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>request_timeout_seconds</t>
+          <t>batch_size</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>120</v>
+        <v>25</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hard limit for each Bloomberg request.</t>
+          <t>Maximum securities sent in one Bloomberg request.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>request_timeout_seconds</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>120</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hard limit for each Bloomberg request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>standalone_max_mb</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B15" t="n">
         <v>20</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Maximum portable HTML size before publication stops.</t>
         </is>

</xml_diff>

<commit_message>
Fix Bloomberg ticker history and export parity
</commit_message>
<xml_diff>
--- a/config/security_roots.xlsx
+++ b/config/security_roots.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Roots" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bloomberg Update" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Security Roots" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bloomberg Update" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Security Roots'!$A$1:$M$8</definedName>
@@ -583,7 +583,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RVO uses Flat with {root} {yellow_key}; Bloomberg pulls RVO Index once and the dashboard applies each daily value across the full curve.</t>
+          <t>RVO uses root NAUG008A with Flat and Index; Bloomberg pulls NAUG008A Index once and the dashboard applies each daily value across the full curve.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Use {y} for 6, {yy} for 26, or {year} for 2026. yellow_key independently controls Comdty vs Index.</t>
+          <t>Use {y} for 6, {yy} for 26, or {year} for 2026. If {y} collides across decades, every colliding year automatically expands (for example WUG18 and WUG28). yellow_key independently controls Comdty vs Index.</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>XB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>RBOB</t>
+          <t>RB|RBOB</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RVO</t>
+          <t>NAUG008A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -961,7 +961,7 @@
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>RENEWABLE VOLUME OBLIGATION</t>
+          <t>RVO|RENEWABLE VOLUME OBLIGATION</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2019-01-01</t>
+          <t>2015-01-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1274,11 +1274,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Maximum dated-contract reference retained, normally 1 or 2.</t>
+          <t>Maximum dated-contract reference retained; use 3 with 36-month history.</t>
         </is>
       </c>
     </row>

</xml_diff>